<commit_message>
update paper and more
</commit_message>
<xml_diff>
--- a/count_students.xlsx
+++ b/count_students.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\GitHub\CV\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B56B6E8E-038D-4A53-B664-02A27359A2B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF1D1DDF-99D0-4C4F-B0D9-1C6E7471463F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{152D85A7-6ADB-4D3D-9731-2BD3ABA9C500}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="31">
   <si>
     <t>שנה</t>
   </si>
@@ -125,7 +125,13 @@
     <t>תואר</t>
   </si>
   <si>
-    <t>מחקר מודרך</t>
+    <t>מדעי הנתונים בפסיכולוגיה</t>
+  </si>
+  <si>
+    <t>מבוא לסטטיסטיקה למדעי המוח</t>
+  </si>
+  <si>
+    <t>מחקר מודרך (סטט)</t>
   </si>
 </sst>
 </file>
@@ -497,8 +503,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DA99827-F5F0-41BD-81FC-680D1AE82FB7}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:H50"/>
+  <dimension ref="A1:H58"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="5.140625" bestFit="1" customWidth="1"/>
@@ -536,15 +541,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>2017</v>
+        <v>2015</v>
       </c>
       <c r="B2" t="s">
         <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -553,64 +558,64 @@
         <v>6</v>
       </c>
       <c r="F2">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="G2" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>2018</v>
+        <v>2016</v>
       </c>
       <c r="B3" t="s">
         <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3" t="s">
         <v>6</v>
       </c>
       <c r="F3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2017</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4" t="s">
+        <v>6</v>
+      </c>
+      <c r="F4">
         <v>50</v>
       </c>
-      <c r="G3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>2022</v>
-      </c>
-      <c r="B4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="E4" t="s">
-        <v>9</v>
-      </c>
-      <c r="F4">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>2015</v>
+        <v>2017</v>
       </c>
       <c r="B5" t="s">
         <v>5</v>
       </c>
       <c r="C5" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -619,13 +624,16 @@
         <v>6</v>
       </c>
       <c r="F5">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="G5" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2017</v>
       </c>
@@ -647,11 +655,8 @@
       <c r="G6" t="b">
         <v>1</v>
       </c>
-      <c r="H6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2017</v>
       </c>
@@ -659,62 +664,62 @@
         <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E7" t="s">
         <v>6</v>
       </c>
       <c r="F7">
-        <v>60</v>
-      </c>
-      <c r="G7" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>2020</v>
+        <v>2018</v>
       </c>
       <c r="B8" t="s">
         <v>5</v>
       </c>
       <c r="C8" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E8" t="s">
         <v>6</v>
       </c>
       <c r="F8">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+        <v>50</v>
+      </c>
+      <c r="G8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>2021</v>
+        <v>2018</v>
       </c>
       <c r="B9" t="s">
         <v>5</v>
       </c>
       <c r="C9" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="D9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E9" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F9">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2019</v>
       </c>
@@ -734,15 +739,15 @@
         <v>63</v>
       </c>
     </row>
-    <row r="11" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11">
-        <v>2016</v>
+        <v>2019</v>
       </c>
       <c r="B11" t="s">
         <v>5</v>
       </c>
       <c r="C11" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="D11">
         <v>2</v>
@@ -751,18 +756,18 @@
         <v>6</v>
       </c>
       <c r="F11">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12">
-        <v>2017</v>
+        <v>2020</v>
       </c>
       <c r="B12" t="s">
         <v>5</v>
       </c>
       <c r="C12" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="D12">
         <v>2</v>
@@ -771,12 +776,12 @@
         <v>6</v>
       </c>
       <c r="F12">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="B13" t="s">
         <v>5</v>
@@ -791,18 +796,18 @@
         <v>6</v>
       </c>
       <c r="F13">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="B14" t="s">
         <v>5</v>
       </c>
       <c r="C14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D14">
         <v>2</v>
@@ -811,10 +816,10 @@
         <v>6</v>
       </c>
       <c r="F14">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2021</v>
       </c>
@@ -834,15 +839,15 @@
         <v>64</v>
       </c>
     </row>
-    <row r="16" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="B16" t="s">
         <v>5</v>
       </c>
       <c r="C16" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="D16">
         <v>1</v>
@@ -851,18 +856,18 @@
         <v>9</v>
       </c>
       <c r="F16">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="B17" t="s">
         <v>5</v>
       </c>
       <c r="C17" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="D17">
         <v>1</v>
@@ -871,201 +876,198 @@
         <v>9</v>
       </c>
       <c r="F17">
-        <v>82</v>
+        <v>309</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="B18" t="s">
         <v>5</v>
       </c>
       <c r="C18" t="s">
+        <v>12</v>
+      </c>
+      <c r="D18">
+        <v>2</v>
+      </c>
+      <c r="E18" t="s">
+        <v>9</v>
+      </c>
+      <c r="F18">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>2022</v>
+      </c>
+      <c r="B19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C19" t="s">
         <v>13</v>
       </c>
-      <c r="D18">
-        <v>2</v>
-      </c>
-      <c r="E18" t="s">
-        <v>9</v>
-      </c>
-      <c r="F18">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A19">
-        <v>2023</v>
-      </c>
-      <c r="B19" t="s">
-        <v>5</v>
-      </c>
-      <c r="C19" t="s">
-        <v>19</v>
-      </c>
       <c r="D19">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E19" t="s">
         <v>9</v>
       </c>
       <c r="F19">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="B20" t="s">
         <v>5</v>
       </c>
       <c r="C20" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="D20">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E20" t="s">
         <v>9</v>
       </c>
       <c r="F20">
-        <v>62</v>
+        <v>21</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21">
-        <v>2026</v>
+        <v>2023</v>
       </c>
       <c r="B21" t="s">
         <v>5</v>
       </c>
       <c r="C21" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="D21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E21" t="s">
         <v>9</v>
       </c>
       <c r="F21">
-        <v>11</v>
+        <v>73</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="B22" t="s">
         <v>5</v>
       </c>
       <c r="C22" t="s">
+        <v>19</v>
+      </c>
+      <c r="D22">
+        <v>1</v>
+      </c>
+      <c r="E22" t="s">
+        <v>9</v>
+      </c>
+      <c r="F22">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>2023</v>
+      </c>
+      <c r="B23" t="s">
+        <v>5</v>
+      </c>
+      <c r="C23" t="s">
+        <v>26</v>
+      </c>
+      <c r="D23">
+        <v>1</v>
+      </c>
+      <c r="E23" t="s">
+        <v>9</v>
+      </c>
+      <c r="F23">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>2023</v>
+      </c>
+      <c r="B24" t="s">
+        <v>14</v>
+      </c>
+      <c r="C24" t="s">
         <v>12</v>
       </c>
-      <c r="D22">
-        <v>2</v>
-      </c>
-      <c r="E22" t="s">
-        <v>9</v>
-      </c>
-      <c r="F22">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A23">
-        <v>2018</v>
-      </c>
-      <c r="B23" t="s">
-        <v>5</v>
-      </c>
-      <c r="C23" t="s">
-        <v>25</v>
-      </c>
-      <c r="D23">
-        <v>1</v>
-      </c>
-      <c r="E23" t="s">
-        <v>9</v>
-      </c>
-      <c r="F23">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A24">
-        <v>2022</v>
-      </c>
-      <c r="B24" t="s">
-        <v>5</v>
-      </c>
-      <c r="C24" t="s">
-        <v>26</v>
-      </c>
       <c r="D24">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E24" t="s">
         <v>9</v>
       </c>
       <c r="F24">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2023</v>
       </c>
       <c r="B25" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="C25" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="D25">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E25" t="s">
         <v>9</v>
       </c>
       <c r="F25">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="B26" t="s">
         <v>5</v>
       </c>
       <c r="C26" t="s">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="D26">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E26" t="s">
         <v>9</v>
       </c>
       <c r="F26">
-        <v>3</v>
-      </c>
-      <c r="H26" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2023</v>
       </c>
       <c r="B27" t="s">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="C27" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D27">
         <v>2</v>
@@ -1074,18 +1076,18 @@
         <v>9</v>
       </c>
       <c r="F27">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>2023</v>
       </c>
       <c r="B28" t="s">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="C28" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="D28">
         <v>2</v>
@@ -1094,50 +1096,50 @@
         <v>9</v>
       </c>
       <c r="F28">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="B29" t="s">
         <v>5</v>
       </c>
       <c r="C29" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D29">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E29" t="s">
         <v>9</v>
       </c>
       <c r="F29">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B30" t="s">
         <v>5</v>
       </c>
       <c r="C30" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="D30">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E30" t="s">
         <v>9</v>
       </c>
       <c r="F30">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>2024</v>
       </c>
@@ -1145,27 +1147,30 @@
         <v>5</v>
       </c>
       <c r="C31" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="D31">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E31" t="s">
         <v>9</v>
       </c>
       <c r="F31">
-        <v>12</v>
+        <v>3</v>
+      </c>
+      <c r="H31" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B32" t="s">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="C32" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D32">
         <v>2</v>
@@ -1174,18 +1179,18 @@
         <v>9</v>
       </c>
       <c r="F32">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B33" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="C33" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="D33">
         <v>2</v>
@@ -1194,10 +1199,10 @@
         <v>9</v>
       </c>
       <c r="F33">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>2024</v>
       </c>
@@ -1205,7 +1210,7 @@
         <v>14</v>
       </c>
       <c r="C34" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D34">
         <v>2</v>
@@ -1214,18 +1219,18 @@
         <v>9</v>
       </c>
       <c r="F34">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>2024</v>
       </c>
       <c r="B35" t="s">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="C35" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="D35">
         <v>2</v>
@@ -1237,9 +1242,9 @@
         <v>11</v>
       </c>
     </row>
-    <row r="36" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36">
-        <v>2022</v>
+        <v>2025</v>
       </c>
       <c r="B36" t="s">
         <v>5</v>
@@ -1254,27 +1259,27 @@
         <v>9</v>
       </c>
       <c r="F36">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="B37" t="s">
         <v>5</v>
       </c>
       <c r="C37" t="s">
+        <v>12</v>
+      </c>
+      <c r="D37">
+        <v>2</v>
+      </c>
+      <c r="E37" t="s">
+        <v>9</v>
+      </c>
+      <c r="F37">
         <v>13</v>
-      </c>
-      <c r="D37">
-        <v>2</v>
-      </c>
-      <c r="E37" t="s">
-        <v>9</v>
-      </c>
-      <c r="F37">
-        <v>50</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
@@ -1285,7 +1290,7 @@
         <v>14</v>
       </c>
       <c r="C38" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D38">
         <v>2</v>
@@ -1294,12 +1299,12 @@
         <v>9</v>
       </c>
       <c r="F38">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39">
-        <v>2022</v>
+        <v>2025</v>
       </c>
       <c r="B39" t="s">
         <v>5</v>
@@ -1314,18 +1319,18 @@
         <v>9</v>
       </c>
       <c r="F39">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="B40" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="C40" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="D40">
         <v>2</v>
@@ -1334,18 +1339,18 @@
         <v>9</v>
       </c>
       <c r="F40">
-        <v>9</v>
+        <v>26</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B41" t="s">
         <v>5</v>
       </c>
       <c r="C41" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="D41">
         <v>1</v>
@@ -1354,32 +1359,32 @@
         <v>9</v>
       </c>
       <c r="F41">
-        <v>32</v>
+        <v>70</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42">
+        <v>2025</v>
+      </c>
+      <c r="B42" t="s">
+        <v>5</v>
+      </c>
+      <c r="C42" t="s">
+        <v>10</v>
+      </c>
+      <c r="D42">
+        <v>1</v>
+      </c>
+      <c r="E42" t="s">
+        <v>9</v>
+      </c>
+      <c r="F42">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43">
         <v>2026</v>
-      </c>
-      <c r="B42" t="s">
-        <v>5</v>
-      </c>
-      <c r="C42" t="s">
-        <v>17</v>
-      </c>
-      <c r="D42">
-        <v>2</v>
-      </c>
-      <c r="E42" t="s">
-        <v>9</v>
-      </c>
-      <c r="F42">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A43">
-        <v>2024</v>
       </c>
       <c r="B43" t="s">
         <v>5</v>
@@ -1399,13 +1404,13 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B44" t="s">
         <v>5</v>
       </c>
       <c r="C44" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="D44">
         <v>1</v>
@@ -1414,27 +1419,27 @@
         <v>9</v>
       </c>
       <c r="F44">
-        <v>70</v>
+        <v>32</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B45" t="s">
         <v>5</v>
       </c>
       <c r="C45" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D45">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E45" t="s">
         <v>9</v>
       </c>
       <c r="F45">
-        <v>103</v>
+        <v>58</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
@@ -1453,6 +1458,9 @@
       <c r="E46" t="s">
         <v>9</v>
       </c>
+      <c r="F46">
+        <v>90</v>
+      </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47">
@@ -1470,6 +1478,9 @@
       <c r="E47" t="s">
         <v>9</v>
       </c>
+      <c r="F47">
+        <v>13</v>
+      </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48">
@@ -1487,8 +1498,11 @@
       <c r="E48" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F48">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>2026</v>
       </c>
@@ -1504,8 +1518,11 @@
       <c r="E49" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F49">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>2026</v>
       </c>
@@ -1521,17 +1538,150 @@
       <c r="E50" t="s">
         <v>9</v>
       </c>
+      <c r="F50">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <v>2027</v>
+      </c>
+      <c r="B51" t="s">
+        <v>5</v>
+      </c>
+      <c r="C51" t="s">
+        <v>17</v>
+      </c>
+      <c r="D51">
+        <v>2</v>
+      </c>
+      <c r="E51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>2027</v>
+      </c>
+      <c r="B52" t="s">
+        <v>5</v>
+      </c>
+      <c r="C52" t="s">
+        <v>28</v>
+      </c>
+      <c r="D52">
+        <v>2</v>
+      </c>
+      <c r="E52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>2027</v>
+      </c>
+      <c r="B53" t="s">
+        <v>14</v>
+      </c>
+      <c r="C53" t="s">
+        <v>29</v>
+      </c>
+      <c r="D53">
+        <v>1</v>
+      </c>
+      <c r="E53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <v>2027</v>
+      </c>
+      <c r="B54" t="s">
+        <v>5</v>
+      </c>
+      <c r="C54" t="s">
+        <v>30</v>
+      </c>
+      <c r="D54">
+        <v>1</v>
+      </c>
+      <c r="E54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55">
+        <v>2027</v>
+      </c>
+      <c r="B55" t="s">
+        <v>5</v>
+      </c>
+      <c r="C55" t="s">
+        <v>19</v>
+      </c>
+      <c r="D55">
+        <v>1</v>
+      </c>
+      <c r="E55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56">
+        <v>2027</v>
+      </c>
+      <c r="B56" t="s">
+        <v>5</v>
+      </c>
+      <c r="C56" t="s">
+        <v>13</v>
+      </c>
+      <c r="D56">
+        <v>2</v>
+      </c>
+      <c r="E56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <v>2027</v>
+      </c>
+      <c r="B57" t="s">
+        <v>14</v>
+      </c>
+      <c r="C57" t="s">
+        <v>12</v>
+      </c>
+      <c r="D57">
+        <v>2</v>
+      </c>
+      <c r="E57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <v>2027</v>
+      </c>
+      <c r="B58" t="s">
+        <v>14</v>
+      </c>
+      <c r="C58" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58">
+        <v>2</v>
+      </c>
+      <c r="E58" t="s">
+        <v>9</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:H49" xr:uid="{2DA99827-F5F0-41BD-81FC-680D1AE82FB7}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="2025"/>
-        <filter val="2026"/>
-      </filters>
-    </filterColumn>
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A18:H51">
-      <sortCondition ref="F1:F49"/>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H52">
+      <sortCondition ref="A1:A49"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>